<commit_message>
Refresh stale root README.md against the actual current project
The README still described the original single-map/one-generic-civ/
no-naval prototype and stopped its milestone list at item 26. Rewrote it
to reflect the real current state: 5 civilizations, 4 Ages, ~25 unit
types with tier ladders, naval combat, diplomacy, a scenario editor with
LAN play, and a working LAN multiplayer MVP. Also closed out this item in
the Master Reference workbook.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KingdomsOfBharat_Master_Reference.xlsx
+++ b/docs/KingdomsOfBharat_Master_Reference.xlsx
@@ -31129,7 +31129,7 @@
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="22" t="inlineStr">
         <is>
-          <t>The project's own session protocol is one roadmap item per session, user's call on which. Two items this sheet previously listed as open turned out already closed once checked directly against the repo on 2026-09-14 (portrait display wiring - commit 42a5a2c; the Maurya/Maratha UniqueTechDefinition crash - commit 6c3d21c, with regression tests) - a reminder to verify status against Assets/Scripts before starting, not just this sheet. The natural remaining candidates: (1) pick up Wave 6's decision-free items - idle-worker indicator, cheat codes, tutorial content; (2) resolve the design decisions gating Relics, Wonder/KotH victory conditions and game modes; (3) refresh the confirmed-stale README; (4) unit-side team colour once Blender masks are sourced.</t>
+          <t>The project's own session protocol is one roadmap item per session, user's call on which. Two items this sheet previously listed as open turned out already closed once checked directly against the repo on 2026-09-14 (portrait display wiring - commit 42a5a2c; the Maurya/Maratha UniqueTechDefinition crash - commit 6c3d21c, with regression tests). README.md was refreshed the same day (rewritten from the stale single-map/one-generic-civ prototype description to reflect the actual current project). The natural remaining candidates: (1) pick up Wave 6's decision-free items - idle-worker indicator, cheat codes, tutorial content; (2) resolve the design decisions gating Relics, Wonder/KotH victory conditions and game modes; (3) unit-side team colour once Blender masks are sourced.</t>
         </is>
       </c>
     </row>
@@ -34123,12 +34123,12 @@
       </c>
       <c r="D31" s="56" t="inlineStr">
         <is>
-          <t>[ ] Not Started</t>
+          <t>[OK] Implemented</t>
         </is>
       </c>
       <c r="E31" s="22" t="inlineStr">
         <is>
-          <t>The root README.md still describes the original single-map/3-civ/no-naval prototype scope and stops its milestone list at 26 - confirmed badly stale 2026-09-03. Pure doc-writing, zero blocker.</t>
+          <t>Closed 2026-09-14. Rewritten to reflect the actual current project (5 civs, 4 Ages, ~25-type unit roster with tier ladders, naval, diplomacy, scenario editor with LAN play, LAN multiplayer MVP) instead of the original single-map/one-generic-civ/no-naval prototype.</t>
         </is>
       </c>
       <c r="F31" s="22" t="inlineStr">
@@ -34492,12 +34492,12 @@
       </c>
       <c r="D46" s="56" t="inlineStr">
         <is>
-          <t>[ ] Not Started</t>
+          <t>[OK] Implemented</t>
         </is>
       </c>
       <c r="E46" s="22" t="inlineStr">
         <is>
-          <t>Confirmed stale 2026-09-03; stops its own milestone list at item 26.</t>
+          <t>Closed 2026-09-14 - see row 31 above for detail.</t>
         </is>
       </c>
       <c r="F46" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Wave 6 item 39: cheat codes console (not live-verified)
New Core/CheatCommandParser.cs (pure) + Core/CheatCodes.cs (executor):
resources/wood/food/gold/stone <n>, age <name>, reveal, spawn <unitType>
[count], win, lose, help - always targets FactionId.Player. New
UI/CheatConsole.cs: BackQuote-toggled typed console, same self-bootstrap
pattern as SettingsMenu/HotkeyOverlay, refuses to run while
NetworkMatch.IsActive. Added the two small public hooks neither
FogOfWarManager nor MatchManager had before (ToggleRevealAll/
ForceOutcome). 17 new EditMode tests.

Not live-verified this session: both unity/UnityMCP MCP servers were
unreachable despite a real Editor + bridge process running against this
project. Flagged in CLAUDE.md/SESSION_LOG.md/the roadmap workbook as
needing a follow-up test run + live verification before being treated
as fully closed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KingdomsOfBharat_Master_Reference.xlsx
+++ b/docs/KingdomsOfBharat_Master_Reference.xlsx
@@ -30295,6 +30295,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -30314,6 +30315,7 @@
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="6" t="n"/>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
@@ -30537,6 +30539,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
@@ -30676,6 +30679,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
@@ -30807,6 +30811,7 @@
         <v/>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
@@ -30870,6 +30875,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
@@ -30887,13 +30893,14 @@
     <row r="47" ht="44" customHeight="1">
       <c r="A47" s="22" t="inlineStr">
         <is>
-          <t>- Wave 6 backlog - 7 of 9 items still open, all parallel-safe. The two remaining with no design decision are cheat codes and tutorial content.</t>
+          <t>- Wave 6 backlog - 6 of 9 items still open. Item 39 (Cheat codes) was built 2026-09-15 but is NOT yet live-verified (MCP servers unreachable that session) - treat it as code-complete, not closed, until a test run + live check happens. The two remaining with no design decision are Score system (36) and tutorial content (40).</t>
         </is>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1">
       <c r="A48" s="22" t="n"/>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
@@ -31088,6 +31095,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
@@ -31119,6 +31127,7 @@
     <row r="67" ht="32" customHeight="1">
       <c r="A67" s="22" t="n"/>
     </row>
+    <row r="68"/>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
@@ -31129,7 +31138,7 @@
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="22" t="inlineStr">
         <is>
-          <t>The project's own session protocol is one roadmap item per session, user's call on which. Two items this sheet previously listed as open turned out already closed once checked directly against the repo on 2026-09-14 (portrait display wiring - commit 42a5a2c; the Maurya/Maratha UniqueTechDefinition crash - commit 6c3d21c, with regression tests). README.md was refreshed the same day, and Wave 6 item 34 (idle-worker indicator) was closed the same day too. The natural remaining candidates: (1) pick up another Wave 6 decision-free item - cheat codes, tutorial content; (2) resolve the design decisions gating Relics, Wonder/KotH victory conditions and game modes; (3) unit-side team colour once Blender masks are sourced.</t>
+          <t>The project's own session protocol is one roadmap item per session, user's call on which. Wave 6 item 39 (Cheat codes) was picked up 2026-09-15 but needs a follow-up test run + live UnityMCP verification before it counts as closed (both MCP servers were unreachable that session). The natural remaining candidates: (1) verify item 39, then pick up another Wave 6 decision-free item - Score system, tutorial content; (2) resolve the design decisions gating Relics, Wonder/KotH victory conditions and game modes; (3) unit-side team colour once Blender masks are sourced.</t>
         </is>
       </c>
     </row>
@@ -33192,7 +33201,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="50" t="inlineStr">
         <is>
@@ -34178,7 +34186,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="50" t="inlineStr">
         <is>
@@ -34193,7 +34200,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="50" t="inlineStr">
         <is>
@@ -36790,12 +36796,12 @@
       </c>
       <c r="F43" s="56" t="inlineStr">
         <is>
-          <t>[ ] Not Started</t>
+          <t>[~] Partial - built, not live-verified</t>
         </is>
       </c>
       <c r="G43" s="22" t="inlineStr">
         <is>
-          <t>Low priority, genuinely useful for testing your own scenarios.</t>
+          <t>New Core/CheatCommandParser.cs (pure parser) + Core/CheatCodes.cs (executor, always targets FactionId.Player): resources/wood/food/gold/stone &lt;n&gt;, age &lt;name&gt;, reveal, spawn &lt;unitType&gt; [count], win, lose, help. New UI/CheatConsole.cs (BackQuote hotkey, Quake-style typed console), refuses to run while NetworkMatch.IsActive. Added FogOfWarManager.ToggleRevealAll() and MatchManager.ForceOutcome() as the two small public hooks neither had before. 17 new EditMode tests (Spawn execution not exercised - EntitySpawner hard-errors outside Play mode, same as every other factory caller). NOT LIVE-VERIFIED (2026-09-15) - both unity/UnityMCP MCP servers were unreachable this session despite a real Editor + bridge process running; code was read back against every real API it touches but the EditMode suite was never actually run. Needs a follow-up test run + live verification before being treated as fully closed like every other Wave 6 item.</t>
         </is>
       </c>
       <c r="H43" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Resolve Relics/Wonder/game-modes design decision (Wave 6 items 35/37/38)
Decision-only session, no code: Relics + Monastery collection (economic
gold-trickle only, no new victory condition) and Deathmatch + King of the
Hill game modes are approved; Wonder is declined entirely. Resolved via
AskUserQuestion, recorded in the Master Reference workbook and CLAUDE.md.
Each item is now unblocked and remains its own future one-item-per-session
implementation pickup.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KingdomsOfBharat_Master_Reference.xlsx
+++ b/docs/KingdomsOfBharat_Master_Reference.xlsx
@@ -30887,7 +30887,7 @@
     <row r="47" ht="44" customHeight="1">
       <c r="A47" s="22" t="inlineStr">
         <is>
-          <t>- Wave 6 backlog - every decision-free item is closed as of 2026-09-15 (item 40, Tutorial content, closed the same session as item 36). The 3 remaining open items all need a design decision before any code work: whether Relics/a relic-storage building are wanted at all (35), whether Wonder/KotH victory conditions are wanted (37, gates 38's game modes too).</t>
+          <t>- Wave 6 backlog - every decision-free item is closed as of 2026-09-15 (item 40, Tutorial content, closed the same session as item 36). The 3 remaining open items' design decision was RESOLVED 2026-09-15 (AskUserQuestion, no code written this session): build Relics + Monastery collection (35, economic gold-trickle only, no new victory condition), Deathmatch + King of the Hill game modes (38, KotH IS a new victory condition - see 37), Wonder is explicitly DECLINED (37 stays partial - Time Limit + Regicide closed, Wonder/Relic-victory closed-as-declined, KotH open). Each of Relics/Monastery, Deathmatch, and KotH is its own future one-item-per-session pickup.</t>
         </is>
       </c>
     </row>
@@ -31074,7 +31074,7 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>Relics, Wonder and King-of-the-Hill victory conditions, game modes</t>
+          <t>Relics + Monastery (35), Deathmatch (38), King of the Hill (37/38) - all scoped 2026-09-15, none implemented yet</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -31129,7 +31129,7 @@
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="22" t="inlineStr">
         <is>
-          <t>The project's own session protocol is one roadmap item per session, user's call on which. As of 2026-09-15, every decision-free Wave 6 item is closed (Town Bell, idle-worker indicator, cheat codes, Score system, Tutorial content). What's left: (1) resolve the design decisions gating Relics, Wonder/KotH victory conditions and game modes; (2) unit-side team colour once Blender masks are sourced; (3) UI/art polish or further balance passes, user's call.</t>
+          <t>The project's own session protocol is one roadmap item per session, user's call on which. As of 2026-09-15, every decision-free Wave 6 item is closed (Town Bell, idle-worker indicator, cheat codes, Score system, Tutorial content), AND the Relics/Wonder/game-modes design decision is now resolved (Relics+Monastery economic-only, Deathmatch, King of the Hill; Wonder declined). What's left: (1) implement Relics + Monastery collection (35); (2) implement Deathmatch mode (38); (3) implement King of the Hill zone-control victory (37/38); (4) unit-side team colour once Blender masks are sourced; (5) UI/art polish or further balance passes, user's call.</t>
         </is>
       </c>
     </row>
@@ -36622,7 +36622,7 @@
       </c>
       <c r="E39" s="22" t="inlineStr">
         <is>
-          <t>A yes/no design decision; Wave 4 item 27 if the carrier is Vaidya/Purohita</t>
+          <t>Design decision resolved 2026-09-15 (below); Wave 4 item 27 Monastery already exists as the carrier building</t>
         </is>
       </c>
       <c r="F39" s="56" t="inlineStr">
@@ -36632,7 +36632,7 @@
       </c>
       <c r="G39" s="22" t="inlineStr">
         <is>
-          <t>AoE II relics pay 0.5 gold/sec and can trigger a victory countdown - needs a carrier unit and a building to store them in.</t>
+          <t>DESIGN DECISION RESOLVED 2026-09-15 via AskUserQuestion: build it, economic only. Relics spawn on the map (or drop from destroyed scripted targets), carried by any land unit to a Monastery for a passive Gold trickle (AoE II precedent: 0.5-1x gold/sec per relic garrisoned). Explicitly NO new victory condition tied to relic count/ownership - stays purely economic, keeping scope smaller (user chose "Economic only" over "also add a Relic-count victory option" via AskUserQuestion). Monastery (Wave 4 item 27) is the existing carrier building - no new building needed. Not yet implemented - this was a design-decision-only session, not implementation.</t>
         </is>
       </c>
       <c r="H39" s="22" t="inlineStr">
@@ -36712,7 +36712,7 @@
       </c>
       <c r="G41" s="22" t="inlineStr">
         <is>
-          <t>Time Limit and Regicide are BOTH closed (Regicide pulled forward into Wave 4 item 28's own session, 2026-09-07, opt-in via GameSettings.RegicideEnabled). Wonder and Relic victory conditions remain unbuilt - building all of AoE's victory conditions is not automatically the right scope for this project, flagged as a decision, not an oversight.</t>
+          <t>Time Limit and Regicide are BOTH closed (Regicide pulled forward into Wave 4 item 28's own session, 2026-09-07, opt-in via GameSettings.RegicideEnabled). Wonder and Relic victory conditions remain unbuilt - building all of AoE's victory conditions is not automatically the right scope for this project, flagged as a decision, not an oversight. Wonder is DECLINED as of 2026-09-15 (AskUserQuestion: user did not pick the "Wonder + King-of-the-Hill-style victory" option) - no Wonder building, no Wonder-triggered victory countdown. Relic victory condition also declined (see item 35 - economic only, no new win condition). King of the Hill IS approved as a victory condition, but scoped under item 38 (Game modes) since the user picked it there specifically, not as a Wonder-KotH hybrid.</t>
         </is>
       </c>
       <c r="H41" s="22" t="inlineStr">
@@ -36742,7 +36742,7 @@
       </c>
       <c r="E42" s="22" t="inlineStr">
         <is>
-          <t>Item 37 if modes are tied to specific victory conditions</t>
+          <t>Design decision resolved 2026-09-15 (below)</t>
         </is>
       </c>
       <c r="F42" s="56" t="inlineStr">
@@ -36752,7 +36752,7 @@
       </c>
       <c r="G42" s="22" t="inlineStr">
         <is>
-          <t>Selectable Skirmish/Deathmatch/Regicide-style/Empire-Wars-style modes on top of the scenario system that already exists.</t>
+          <t>DESIGN DECISION RESOLVED 2026-09-15 via AskUserQuestion: build Deathmatch + King of the Hill this wave (not Empire Wars, not asked about). Deathmatch: opt-in GameSettings toggle (same pattern as RegicideEnabled) - match starts with large stockpiles of every resource and a higher starting Age, reusing existing resource-grant/age-set code paths, skips the early economy game. King of the Hill: a map-marked zone; the faction holding it uncontested for N minutes wins - needs a new zone-control tracker and countdown (shape similar to SurviveSeconds objectives but faction-vs-faction and area-based), a genuinely new victory condition (see item 37). Not yet implemented - this was a design-decision-only session; each of Deathmatch/KotH/Relic-Monastery is its own future one-item-per-session pickup per this project's own protocol.</t>
         </is>
       </c>
       <c r="H42" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Decimate age-tiered TownCenter/Tower/Wall building models
Extends the 2026-09-02 mesh-decimation pass (which only covered the 45
Imperial-tier civ-specific buildings) to the age-tiered variants
(Ancient/Classical/Durg), which shipped un-decimated at ~1.9-3.0M tris even
after that pass landed, and again when the 2026-09-15 regression fix
restored them. Caps all reachable targets at the same ~500,000-tri ceiling;
Wall_Durg is skipped and flagged (corrupted shared source FBX, unrelated to
this work) rather than crashing the batch. 581/581 EditMode tests pass;
live-verified via UnityMCP through the real BuildingModelFactory.Spawn path.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KingdomsOfBharat_Master_Reference.xlsx
+++ b/docs/KingdomsOfBharat_Master_Reference.xlsx
@@ -30270,7 +30270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -30866,7 +30866,7 @@
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="22" t="inlineStr">
         <is>
-          <t>- UI: ornate HUD art pass (UI_ART_BRIEF Tiers 1-3), AoE-style single bottom bar, paginated icon command grid with tooltips, group-selection icon row, an always-visible Age/research meter, and (2026-09-14) SelectedUnitPanel portrait display wiring for the 21 generic-unit portraits, including TradeShipFactory's IconKey.</t>
+          <t>- UI: ornate HUD art pass (UI_ART_BRIEF Tiers 1-3), AoE-style single bottom bar, paginated icon command grid with tooltips, group-selection icon row, an always-visible Age/research meter, and (2026-09-14) SelectedUnitPanel portrait display wiring for the 21 generic-unit portraits, including TradeShipFactory's IconKey. (2026-09-16) Age-tiered TownCenter/Tower/Wall models (Ancient/Classical/Durg) decimated to the same ~500,000-tri ceiling as the 45 Imperial-tier models, except Wall_Durg (corrupted shared source, see Blocked table).</t>
         </is>
       </c>
     </row>
@@ -31038,98 +31038,117 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>Fish Trap</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>Art sourcing</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>The Farm half of the renewable-resource item closed 2026-09-03; the Fish Trap half was never started.</t>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Wall_Durg model (shared, all 5 civs)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Corrupted source FBX</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Reports 0 vertices/bounds while triangles.Length still claims ~3.08M stale indices - reproduced on a fresh-GUID copy, ruling out cache/import causes. Needs a re-exported source; currently spawns un-decimated via the existing fallback chain.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Store / marketing assets</t>
+          <t>Fish Trap</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>A user decision</t>
+          <t>Art sourcing</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Needs an explicit ruling on whether public release is a goal before it can even be scoped.</t>
+          <t>The Farm half of the renewable-resource item closed 2026-09-03; the Fish Trap half was never started.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
+          <t>Store / marketing assets</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>A user decision</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Needs an explicit ruling on whether public release is a goal before it can even be scoped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
           <t>Relics + Monastery (35), Deathmatch (38), King of the Hill (37/38) - all scoped 2026-09-15, none implemented yet</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>A design decision</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Building all of AoE's victory conditions is not automatically the right scope for this project - flagged as a decision, not an oversight.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+    <row r="63"/>
+    <row r="64" ht="32" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>KNOWN OPEN BUGS AND RISKS</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="32" customHeight="1">
-      <c r="A64" s="22" t="inlineStr">
-        <is>
-          <t>- Two pre-existing BuildingModelFactoryTests failures (Chola TownCenter model) are the stable baseline in every recent session - 520 of 522 EditMode tests pass.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="32" customHeight="1">
       <c r="A65" s="22" t="inlineStr">
         <is>
-          <t>- A second, concurrent session was observed committing to this same branch on 2026-09-14. Re-check git status before every commit.</t>
+          <t>- The 2 previously-standing BuildingModelFactoryTests failures (Chola TownCenter model) are gone as of 2026-09-16 - 581/581 EditMode tests pass, up from 520/522.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="32" customHeight="1">
       <c r="A66" s="22" t="inlineStr">
         <is>
+          <t>- A second, concurrent session was observed committing to this same branch on 2026-09-14. Re-check git status before every commit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="32" customHeight="1">
+      <c r="A67" s="22" t="inlineStr">
+        <is>
           <t>- Recurring environment traps worth knowing: Unity's MCP console bridge can report zero errors while code genuinely fails to compile (check ~/Library/Logs/Unity/Editor.log directly), and exiting Play mode does not itself trigger a domain reload, so static state can bleed into the next EditMode run.</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="32" customHeight="1">
-      <c r="A67" s="22" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="22" t="n"/>
+    </row>
+    <row r="69"/>
+    <row r="70" ht="60" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>WHAT'S NEXT (pointer, not a commitment)</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="60" customHeight="1">
-      <c r="A70" s="22" t="inlineStr">
-        <is>
-          <t>The project's own session protocol is one roadmap item per session, user's call on which. As of 2026-09-15, every decision-free Wave 6 item is closed (Town Bell, idle-worker indicator, cheat codes, Score system, Tutorial content), AND the Relics/Wonder/game-modes design decision is now resolved (Relics+Monastery economic-only, Deathmatch, King of the Hill; Wonder declined). What's left: (1) implement Relics + Monastery collection (35); (2) implement Deathmatch mode (38); (3) implement King of the Hill zone-control victory (37/38); (4) unit-side team colour once Blender masks are sourced; (5) UI/art polish or further balance passes, user's call.</t>
+    <row r="71">
+      <c r="A71" s="22" t="inlineStr">
+        <is>
+          <t>The project's own session protocol is one roadmap item per session, user's call on which. As of 2026-09-15, every decision-free Wave 6 item is closed (Town Bell, idle-worker indicator, cheat codes, Score system, Tutorial content), AND the Relics/Wonder/game-modes design decision is now resolved (Relics+Monastery economic-only, Deathmatch, King of the Hill; Wonder declined). Age-tiered building mesh decimation (the last flagged follow-up from the 2026-09-15 regression fix) closed 2026-09-16. What's left: (1) implement Relics + Monastery collection (35); (2) implement Deathmatch mode (38); (3) implement King of the Hill zone-control victory (37/38); (4) unit-side team colour once Blender masks are sourced; (5) UI/art polish or further balance passes, user's call.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add wall drag-placement (Session A) and corner mesh splitting (Session B, in progress)
Session A: mouse-down/drag/mouse-up free-angle placement of Wall segment
chains via BuildingPlacer.ComputeWallChain, with rotation support wired
through WallFactory.Place, CommandSerializer, and NetMessageEnvelope.
9 new EditMode tests, live-verified via UnityMCP.

Session B (in progress): new WallPieceMeshSplitter editor tool does real
geometric plane-clipping to split fused corner meshes into reusable
Pillar + Arm sub-meshes for future auto-tiling. Durg and Ancient tiers
split and screenshot-verified clean; Classical and per-civ Imperial
tiers remain.
</commit_message>
<xml_diff>
--- a/docs/KingdomsOfBharat_Master_Reference.xlsx
+++ b/docs/KingdomsOfBharat_Master_Reference.xlsx
@@ -234,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -360,6 +360,7 @@
     <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -31105,7 +31106,6 @@
         </is>
       </c>
     </row>
-    <row r="63"/>
     <row r="64" ht="32" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
@@ -31137,7 +31137,6 @@
     <row r="68">
       <c r="A68" s="22" t="n"/>
     </row>
-    <row r="69"/>
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
@@ -32042,7 +32041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -32639,7 +32638,7 @@
       </c>
       <c r="C34" s="22" t="inlineStr">
         <is>
-          <t>a South Asian light-armored archer specialized against archers, quilted cotton armor, small round buckler shield strapped to the forearm, short recurve bow and quiver, neutral A-pose, front view. [STATUS: not sourced, reuses shared Archer body]</t>
+          <t>a bare, GEARLESS South Asian light-infantry body built for a fast skirmishing archer - lean/agile build, simple quilted cotton undergarment only (thin padded gambeson, no armor plates, no metal), bare head with no helmet, hands empty and relaxed with no shield or bow modeled onto the mesh. Helmet, forearm buckler, and bow are separate equippable game-asset props attached at runtime via bone sockets from the per-civ gear system (WeaponAttachment.cs), not baked into this body. Neutral A-pose, front and side view for a game character turnaround. [STATUS: not sourced - corrected 2026-09-16 to a gearless base body; reuses the shared Archer body rig, with helmet/shield/bow equipped separately per civ rather than baked into the model]</t>
         </is>
       </c>
     </row>
@@ -32813,10 +32812,18 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="59" t="inlineStr">
+        <is>
+          <t>RULE (corrected 2026-09-16): every new-unit HUMAN CHARACTER body (e.g. Skirmisher above, and the Maharaja hero below) must be sourced GEARLESS - no helmet, shield, or weapon baked onto the mesh. Helmet/shield/weapon are always separate equippable props attached at runtime via bone sockets (WeaponAttachment.AttachToBone), per the 'Per-civ unit gear' table above. Mount-only/machine-only/hull-only assets (Scout horse, Battering Ram, Scorpion, Fire Ship, etc.) are unaffected - they carry no character gear at all.</t>
+        </is>
+      </c>
+    </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="36" t="inlineStr">
         <is>
-          <t>Maharaja hero - one prompt per civilization (Wave 4 item 28, per-civ - shipped, all reuse shared body)</t>
+          <t>Maharaja hero (Wave 4 item 28) - ONE shared GEARLESS hero base body (prompt below) + a per-civ 'Royal/Hero tier' gear set (crown, ceremonial shield, ceremonial sword) in the table below, corrected 2026-09-16. The previous version baked each civ's ornate regalia directly onto 5 separate full-body models, which conflicts with the per-civ gear attachment system (item 5) this project actually uses - fixed to match that system instead.
+Shared hero base body prompt: "a bare, GEARLESS South Asian hero figure on foot, taller and more heroic build than the standard soldier body, simple unadorned royal undergarment/robe base layer only (no armor plates, no crown/helmet, no weapon or shield modeled onto the mesh) - crown, ceremonial armor accents, and ceremonial weapon/shield are separate equippable props attached at runtime via bone sockets, per civ, from the Royal/Hero gear table below. Regal neutral A-pose, front view." [Reused as one shared rig across all 5 civs; only the equipped Royal-tier gear differs per civ, exactly like the standard soldier per-civ gear table above.]</t>
         </is>
       </c>
       <c r="B46" s="37" t="n"/>
@@ -32832,12 +32839,24 @@
       </c>
       <c r="B47" s="38" t="inlineStr">
         <is>
-          <t>Prompt</t>
-        </is>
-      </c>
-      <c r="C47" s="38" t="inlineStr"/>
-      <c r="D47" s="38" t="inlineStr"/>
-      <c r="E47" s="38" t="inlineStr"/>
+          <t>Royal Helmet / Crown</t>
+        </is>
+      </c>
+      <c r="C47" s="38" t="inlineStr">
+        <is>
+          <t>Ceremonial Shield</t>
+        </is>
+      </c>
+      <c r="D47" s="38" t="inlineStr">
+        <is>
+          <t>Ceremonial Weapon</t>
+        </is>
+      </c>
+      <c r="E47" s="38" t="inlineStr">
+        <is>
+          <t>Full prompt</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="75" customHeight="1">
       <c r="A48" s="39" t="inlineStr">
@@ -32847,7 +32866,22 @@
       </c>
       <c r="B48" s="22" t="inlineStr">
         <is>
-          <t>a South Asian Chola Maharaja hero on foot, richly ornate ceremonial armor with bronze relief work and temple-gopuram motifs, royal crown/ceremonial helmet with Nandi-bull or lotus finial, ceremonial sword with bronze basket-hilt, rich royal robes, regal neutral A-pose, front view - the single most elaborate figure of this civilization.</t>
+          <t>Ornate bronze crown, Nandi-bull or lotus finial</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Ceremonial shield, temple-gopuram motif bronze relief rim</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Ceremonial curved sword (patta-style), bronze basket-hilt, rope-motif engraving</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>a separate equippable Royal-tier gear set for the Chola Maharaja - ornate bronze crown with Nandi-bull/lotus finial, ceremonial shield with temple-gopuram motif bronze relief rim, ceremonial patta-style sword with bronze basket-hilt and rope-motif engraving, three separate equippable game-asset props on a plain background, front and side view each - grander than the civ's Imperial-tier soldier gear but the same attachment convention.</t>
         </is>
       </c>
     </row>
@@ -32859,7 +32893,22 @@
       </c>
       <c r="B49" s="22" t="inlineStr">
         <is>
-          <t>richly ornate ceremonial armor with gold and granite-toned accents, elephant-and-lotus relief motifs, royal crown with elephant-tusk crest motif, ceremonial sword with mandapa-pillar-fluted hilt, rich royal robes, regal neutral A-pose, front view.</t>
+          <t>Crown with full elephant-tusk crest motif, gold accents</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Ceremonial shield, full elephant-and-lotus relief medallion, gold/granite tones</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Ceremonial sword with mandapa-pillar-fluted gilt hilt</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>a separate equippable Royal-tier gear set for the Vijayanagara Maharaja - crown with full elephant-tusk crest and gold accents, ceremonial shield with elephant-and-lotus relief medallion in gold/granite tones, ceremonial sword with mandapa-pillar-fluted gilt hilt, three separate equippable game-asset props on a plain background, front and side view each - grander than the civ's Imperial-tier soldier gear but the same attachment convention.</t>
         </is>
       </c>
     </row>
@@ -32871,7 +32920,22 @@
       </c>
       <c r="B50" s="22" t="inlineStr">
         <is>
-          <t>richly ornate ceremonial armor in rose-pink and gilt tones with jharokha-lattice engraving, royal crown/turban with full chhatri-dome crest and plume, ceremonial talwar/katar with gilt hilt and floral chasing, rich royal robes, regal neutral A-pose, front view.</t>
+          <t>Ornate crown/turban, full chhatri-dome crest and plume, gilt trim</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Ceremonial shield, painted jharokha-lattice medallion, rose-pink and gilt accents</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Ceremonial talwar or katar, gilt hilt, floral chasing</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>a separate equippable Royal-tier gear set for the Rajput Maharaja - ornate crown/turban with full chhatri-dome crest, plume, and gilt trim, ceremonial shield with painted jharokha-lattice medallion in rose-pink and gilt, ceremonial talwar/katar with gilt hilt and floral chasing, three separate equippable game-asset props on a plain background, front and side view each - grander than the civ's Imperial-tier soldier gear but the same attachment convention.</t>
         </is>
       </c>
     </row>
@@ -32883,7 +32947,22 @@
       </c>
       <c r="B51" s="22" t="inlineStr">
         <is>
-          <t>richly ornate mirror-polished ceremonial armor, royal crown crested with full four-lion Ashokan capital, ceremonial sword with lion-headed pommel, rich royal robes, regal neutral A-pose, front view.</t>
+          <t>Mirror-polished crown, full four-lion Ashokan capital crest</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Ceremonial shield, stupa-dome medallion and lion motif, mirror-polished trim</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Ceremonial sword with lion-headed pommel</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>a separate equippable Royal-tier gear set for the Maurya Maharaja - mirror-polished crown with full four-lion Ashokan capital crest, ceremonial shield with stupa-dome medallion and lion motif in mirror-polished trim, ceremonial sword with lion-headed pommel, three separate equippable game-asset props on a plain background, front and side view each - grander than the civ's Imperial-tier soldier gear but the same attachment convention.</t>
         </is>
       </c>
     </row>
@@ -32895,14 +32974,29 @@
       </c>
       <c r="B52" s="22" t="inlineStr">
         <is>
-          <t>ceremonial armor deliberately more restrained than other civs' heroes per Maratha's hill-fort identity - dark iron and leather with saffron-and-black royal accents rather than heavy gilding, modest crowned helmet with saffron plume, ceremonial firangi-style sword with saffron-and-black hilt wrap, regal but understated, front view.</t>
+          <t>Dark-iron crowned helmet, saffron-accented plume</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Ceremonial shield, hill-fort bastion motif, saffron-and-black trim</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Ceremonial curved sword (firangi-style), saffron-and-black hilt wrap</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>a separate equippable Royal-tier gear set for the Maratha Maharaja - deliberately understated per the civ's hill-fort identity: dark-iron crowned helmet with saffron-accented plume, ceremonial shield with hill-fort bastion motif and saffron-and-black trim, ceremonial firangi-style sword with saffron-and-black hilt wrap, three separate equippable game-asset props on a plain background, front and side view each - still more ornate than the civ's own Imperial-tier soldier gear, but restrained compared to every other civ's Royal tier.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="45" customHeight="1">
       <c r="A54" s="22" t="inlineStr">
         <is>
-          <t>STATUS: implemented (Wave 4 item 28, 2026-09-07) - but no dedicated per-civ Maharaja model was ever sourced from these prompts; every civ's Maharaja reuses the shared Human Character Dummy + Horse + Sword combo (same as Rajput Royal Guard), visually identical to a Cavalry/Royal-Guard hybrid.</t>
+          <t>STATUS: implemented (Wave 4 item 28, 2026-09-07) using the shared Human Character Dummy + Horse + Sword combo (no dedicated hero model sourced) - visually identical to a Cavalry/Royal-Guard hybrid today. The prompts above were corrected 2026-09-16 (gearless shared hero body + per-civ Royal-tier gear, replacing 5 fully-baked ornate bodies) for whenever a dedicated Maharaja model is actually sourced.</t>
         </is>
       </c>
     </row>
@@ -33024,7 +33118,7 @@
     <row r="63" ht="60" customHeight="1">
       <c r="A63" s="39" t="inlineStr">
         <is>
-          <t>New-unit human characters (Skirmisher, Vaidya, Purohita)</t>
+          <t>New-unit human characters (Skirmisher, Vaidya, Purohita) - GEARLESS bodies; helmet/shield/weapon props use the per-civ gear poly target above</t>
         </is>
       </c>
       <c r="B63" s="22" t="inlineStr">
@@ -33109,7 +33203,7 @@
     <row r="68" ht="60" customHeight="1">
       <c r="A68" s="39" t="inlineStr">
         <is>
-          <t>Maharaja hero (per civ, solo figure)</t>
+          <t>Maharaja hero base body (shared, GEARLESS, per civ Royal-tier gear equipped separately - see per-civ gear poly target above for those props)</t>
         </is>
       </c>
       <c r="B68" s="22" t="inlineStr">
@@ -33119,7 +33213,7 @@
       </c>
       <c r="C68" s="22" t="inlineStr">
         <is>
-          <t>6,000-10,000 tris</t>
+          <t>2,500-4,500 tris (bare body only, taller/heroic build vs. standard soldier); Royal-tier gear props 200-600 tris each</t>
         </is>
       </c>
     </row>
@@ -33140,40 +33234,327 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="36" t="inlineStr">
+        <is>
+          <t>Wall System Session B: Corner &amp; End-Cap pieces (auto-tiling art, added 2026-09-16)</t>
+        </is>
+      </c>
+      <c r="B71" s="36" t="n"/>
+      <c r="C71" s="36" t="n"/>
+      <c r="D71" s="36" t="n"/>
+      <c r="E71" s="36" t="n"/>
+    </row>
+    <row r="72" ht="45" customHeight="1">
+      <c r="A72" s="22" t="inlineStr">
+        <is>
+          <t>Ready-to-paste Gemini prompts for the corner/end-cap pieces Session B (drag-placement wall auto-tiling - see CLAUDE.md's matching status entry and the Roadmap - Open Items sheet) needs before it can be built. Matches the exact style-anchor convention at the top of this sheet and the isolated-object/three-quarter-isometric/plain-background convention already used for every other building concept image in this project. Once generated, convert each through Meshy AI same as every other sourced building asset, then hand the FBX/albedo/normal/metallicSmoothness files back for wiring via BuildingMeshDecimator.cs/MeshyBuildingImporter.cs. NOTE (2026-09-16, user-supplied reference images confirmed the corner design): the corner piece's own pillar/post region can likely be extracted (via triangle-cluster mesh-splitting, no Blender needed) and reused directly as the End-Cap piece, matching AoE's real Pillar+Plank asset convention - the End-Cap prompts below may turn out unnecessary once the real corner mesh is in hand and checked; hold off generating them until that's confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="38" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B74" s="38" t="inlineStr">
+        <is>
+          <t>Piece</t>
+        </is>
+      </c>
+      <c r="C74" s="38" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="90" customHeight="1">
+      <c r="A75" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B75" s="39" t="inlineStr">
+        <is>
+          <t>Wall Corner - Ancient (shared, wooden palisade)</t>
+        </is>
+      </c>
+      <c r="C75" s="22" t="inlineStr">
+        <is>
+          <t>Fortification wall corner concept art for a historical real-time strategy video game. A single isolated 90-degree wall corner/turn piece in a three-quarter isometric view, centered and fully visible on a plain neutral light background. Matches an existing straight wall segment made of sharpened wooden stakes lashed together with rope and leather bindings at intervals, uneven stake heights with pointed tops, sitting on a low rough stone-and-rubble foundation course. The corner piece shows two wall faces meeting at a right angle, with the same stake density and lashing detail continuing around the turn - not two straight segments crudely overlapped. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="90" customHeight="1">
+      <c r="A76" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="B76" s="39" t="inlineStr">
+        <is>
+          <t>Wall Corner - Classical (shared, fieldstone)</t>
+        </is>
+      </c>
+      <c r="C76" s="22" t="inlineStr">
+        <is>
+          <t>Fortification wall corner concept art for a historical real-time strategy video game. A single isolated 90-degree wall corner/turn piece in a three-quarter isometric view, centered and fully visible on a plain neutral light background. Matches an existing straight wall segment built from irregular stacked fieldstone blocks in uneven weathered grey-brown coursing, with a slightly raised rough parapet lip along the top edge. The corner piece shows two wall faces meeting at a right angle with a genuine interlocking quoin-style stone bond at the turn (alternating overlap, like real masonry corners), not two flat segments butted together. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="90" customHeight="1">
+      <c r="A77" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="B77" s="39" t="inlineStr">
+        <is>
+          <t>Wall Corner - Durg (shared, stone rampart)</t>
+        </is>
+      </c>
+      <c r="C77" s="22" t="inlineStr">
+        <is>
+          <t>Fortification wall corner concept art for a historical real-time strategy video game. A single isolated 90-degree wall corner/turn piece in a three-quarter isometric view, centered and fully visible on a plain neutral light background. Matches an existing straight wall segment built from neat courses of cut dressed stone blocks, with a slightly battered (inward-sloping) base, pillared bastion-style pilasters at intervals, narrow arrow-slit apertures along the upper band, and rectangular crenellations/merlons along the top edge. The corner piece shows a reinforced pillared bastion turret exactly at the 90-degree turn where the two wall faces meet, matching the pilaster style already on the straight segment. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="90" customHeight="1">
+      <c r="A78" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="B78" s="39" t="inlineStr">
+        <is>
+          <t>Wall Corner - Chola (Imperial)</t>
+        </is>
+      </c>
+      <c r="C78" s="22" t="inlineStr">
+        <is>
+          <t>Chola civilization Wall Corner building concept art for a historical real-time strategy video game. A single isolated 90-degree wall corner/turn piece in a three-quarter isometric view, centered and fully visible on a plain neutral light background, inspired by Dravidian temple architecture - granite and sandstone construction, stepped pyramidal gopuram-tower motifs, tiered stone terraces, and intricate carved relief work. The corner piece shows two fortification wall faces meeting at a right angle with matching carved stonework and tiered detailing continuing around the turn. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="90" customHeight="1">
+      <c r="A79" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B79" s="39" t="inlineStr">
+        <is>
+          <t>Wall Corner - Vijayanagara (Imperial)</t>
+        </is>
+      </c>
+      <c r="C79" s="22" t="inlineStr">
+        <is>
+          <t>Vijayanagara civilization Wall Corner building concept art for a historical real-time strategy video game. A single isolated 90-degree wall corner/turn piece in a three-quarter isometric view, centered and fully visible on a plain neutral light background, inspired by Hampi-style Deccan architecture - monolithic weathered grey-brown granite blockwork, elephant and lotus relief carvings, and a flat corbelled roofline. The corner piece shows two fortification wall faces meeting at a right angle with matching granite blockwork and relief carving continuing around the turn. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="90" customHeight="1">
+      <c r="A80" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="B80" s="39" t="inlineStr">
+        <is>
+          <t>Wall Corner - Rajput (Imperial)</t>
+        </is>
+      </c>
+      <c r="C80" s="22" t="inlineStr">
+        <is>
+          <t>Rajput civilization Wall Corner building concept art for a historical real-time strategy video game. A single isolated 90-degree wall corner/turn piece in a three-quarter isometric view, centered and fully visible on a plain neutral light background, inspired by fort-and-haveli architecture - rose-pink sandstone walls, a domed chhatri pavilion at the corner, ornately latticed jharokha detailing, and a crenellated rampart parapet. The corner piece shows two fortification wall faces meeting at a right angle beneath the corner chhatri dome. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="90" customHeight="1">
+      <c r="A81" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="B81" s="39" t="inlineStr">
+        <is>
+          <t>Wall Corner - Maurya (Imperial)</t>
+        </is>
+      </c>
+      <c r="C81" s="22" t="inlineStr">
+        <is>
+          <t>Mauryan imperial Wall Corner building concept art for a historical real-time strategy video game. A single isolated 90-degree wall corner/turn piece in a three-quarter isometric view, centered and fully visible on a plain neutral light background, inspired by Mauryan imperial architecture - polished cream Chunar sandstone with the famous Mauryan mirror-shine finish, lion-capital pillar motifs, and restrained massive geometric forms. The corner piece shows two fortification wall faces meeting at a right angle with matching polished sandstone and pillar detailing continuing around the turn. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="90" customHeight="1">
+      <c r="A82" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="B82" s="39" t="inlineStr">
+        <is>
+          <t>Wall Corner - Maratha (Imperial)</t>
+        </is>
+      </c>
+      <c r="C82" s="22" t="inlineStr">
+        <is>
+          <t>Maratha civilization Wall Corner building concept art for a historical real-time strategy video game. A single isolated 90-degree wall corner/turn piece in a three-quarter isometric view, centered and fully visible on a plain neutral light background, inspired by Deccan hill-fort architecture - rugged dark basalt stone construction, battered sloped bastion walls, a squat corner watch-burj, and minimal ornamentation, built for function over display. The corner piece shows a squat watch-burj bastion exactly at the 90-degree turn where the two wall faces meet. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="90" customHeight="1">
+      <c r="A83" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="B83" s="39" t="inlineStr">
+        <is>
+          <t>Wall End-Cap - Ancient (shared, wooden palisade)</t>
+        </is>
+      </c>
+      <c r="C83" s="22" t="inlineStr">
+        <is>
+          <t>Fortification wall end-cap concept art for a historical real-time strategy video game. A single isolated wall end-cap piece - where a wall line terminates cleanly - in a three-quarter isometric view, centered and fully visible on a plain neutral light background. Matches an existing straight wall segment made of sharpened wooden stakes lashed together with rope and leather bindings, sitting on a low rough stone-and-rubble foundation. The terminal end is capped by a single stouter squared timber post, slightly taller than the surrounding stakes and with visible rope lashing wrapped around its top, so the wall clearly reads as deliberately ending rather than being cut off mid-structure. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="90" customHeight="1">
+      <c r="A84" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="B84" s="39" t="inlineStr">
+        <is>
+          <t>Wall End-Cap - Classical (shared, fieldstone)</t>
+        </is>
+      </c>
+      <c r="C84" s="22" t="inlineStr">
+        <is>
+          <t>Fortification wall end-cap concept art for a historical real-time strategy video game. A single isolated wall end-cap piece - where a wall line terminates cleanly - in a three-quarter isometric view, centered and fully visible on a plain neutral light background. Matches an existing straight wall segment built from irregular stacked fieldstone blocks in uneven weathered grey-brown coursing. The terminal end is capped by a solid squared stone pier slightly thicker than the wall itself, with a small flat stone cap on top, so it reads as a finished stub rather than broken masonry. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="90" customHeight="1">
+      <c r="A85" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="B85" s="39" t="inlineStr">
+        <is>
+          <t>Wall End-Cap - Durg (shared, stone rampart)</t>
+        </is>
+      </c>
+      <c r="C85" s="22" t="inlineStr">
+        <is>
+          <t>Fortification wall end-cap concept art for a historical real-time strategy video game. A single isolated wall end-cap piece - where a wall line terminates cleanly - in a three-quarter isometric view, centered and fully visible on a plain neutral light background. Matches an existing straight wall segment built from neat courses of cut dressed stone with pillared bastion-style pilasters and rectangular crenellations. The terminal end is capped by one of the wall's own pillared bastion pilasters, matching the corner piece's pilaster style, with a single merlon centered on the flat terminal face. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="90" customHeight="1">
+      <c r="A86" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="B86" s="39" t="inlineStr">
+        <is>
+          <t>Wall End-Cap - Chola (Imperial)</t>
+        </is>
+      </c>
+      <c r="C86" s="22" t="inlineStr">
+        <is>
+          <t>Chola civilization Wall End-Cap building concept art for a historical real-time strategy video game. A single isolated wall end-cap piece - where a fortification wall line terminates cleanly - in a three-quarter isometric view, centered and fully visible on a plain neutral light background, inspired by Dravidian temple architecture. The terminal end is capped by a small stepped gopuram-finial post matching the wall's own granite and sandstone carved-relief style. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="90" customHeight="1">
+      <c r="A87" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="B87" s="39" t="inlineStr">
+        <is>
+          <t>Wall End-Cap - Vijayanagara (Imperial)</t>
+        </is>
+      </c>
+      <c r="C87" s="22" t="inlineStr">
+        <is>
+          <t>Vijayanagara civilization Wall End-Cap building concept art for a historical real-time strategy video game. A single isolated wall end-cap piece - where a fortification wall line terminates cleanly - in a three-quarter isometric view, centered and fully visible on a plain neutral light background, inspired by Hampi-style Deccan architecture. The terminal end is capped by a monolithic granite pillar stub with a carved lotus finial, matching the wall's own weathered grey-brown blockwork. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="90" customHeight="1">
+      <c r="A88" s="22" t="n">
+        <v>14</v>
+      </c>
+      <c r="B88" s="39" t="inlineStr">
+        <is>
+          <t>Wall End-Cap - Rajput (Imperial)</t>
+        </is>
+      </c>
+      <c r="C88" s="22" t="inlineStr">
+        <is>
+          <t>Rajput civilization Wall End-Cap building concept art for a historical real-time strategy video game. A single isolated wall end-cap piece - where a fortification wall line terminates cleanly - in a three-quarter isometric view, centered and fully visible on a plain neutral light background, inspired by fort-and-haveli architecture. The terminal end is capped by a small chhatri-domed post in rose-pink sandstone, matching the wall's own jharokha-latticed style. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="90" customHeight="1">
+      <c r="A89" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="B89" s="39" t="inlineStr">
+        <is>
+          <t>Wall End-Cap - Maurya (Imperial)</t>
+        </is>
+      </c>
+      <c r="C89" s="22" t="inlineStr">
+        <is>
+          <t>Mauryan imperial Wall End-Cap building concept art for a historical real-time strategy video game. A single isolated wall end-cap piece - where a fortification wall line terminates cleanly - in a three-quarter isometric view, centered and fully visible on a plain neutral light background, inspired by Mauryan imperial architecture. The terminal end is capped by a polished cream Chunar sandstone pillar stub with a small lion-capital cap, matching the wall's own mirror-shine finish. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="90" customHeight="1">
+      <c r="A90" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="B90" s="39" t="inlineStr">
+        <is>
+          <t>Wall End-Cap - Maratha (Imperial)</t>
+        </is>
+      </c>
+      <c r="C90" s="22" t="inlineStr">
+        <is>
+          <t>Maratha civilization Wall End-Cap building concept art for a historical real-time strategy video game. A single isolated wall end-cap piece - where a fortification wall line terminates cleanly - in a three-quarter isometric view, centered and fully visible on a plain neutral light background, inspired by Deccan hill-fort architecture. The terminal end is capped by a squat dark-basalt watch-post, deliberately unornamented, matching the wall's own rugged battered-stone style. No other buildings, characters, ground clutter, or scenery in the shot. [STATUS: NOT STARTED - Session B (wall auto-tiling), needs Gemini generation + Meshy AI conversion, then wire via BuildingMeshDecimator/MeshyBuildingImporter same as every other building asset]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="44">
     <mergeCell ref="C44:E44"/>
     <mergeCell ref="C41:E41"/>
-    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="C84:E84"/>
     <mergeCell ref="C40:E40"/>
-    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="C90:E90"/>
     <mergeCell ref="C59:E59"/>
     <mergeCell ref="C43:E43"/>
     <mergeCell ref="C60:E60"/>
     <mergeCell ref="C65:E65"/>
     <mergeCell ref="C36:E36"/>
-    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="C76:E76"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="C39:E39"/>
+    <mergeCell ref="C82:E82"/>
     <mergeCell ref="C67:E67"/>
+    <mergeCell ref="C81:E81"/>
     <mergeCell ref="C38:E38"/>
     <mergeCell ref="C66:E66"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="C37:E37"/>
-    <mergeCell ref="B52:E52"/>
-    <mergeCell ref="B48:E48"/>
     <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C87:E87"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="C86:E86"/>
     <mergeCell ref="C68:E68"/>
+    <mergeCell ref="C77:E77"/>
     <mergeCell ref="C34:E34"/>
+    <mergeCell ref="C83:E83"/>
     <mergeCell ref="C62:E62"/>
     <mergeCell ref="C42:E42"/>
     <mergeCell ref="C58:E58"/>
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="A4:E4"/>
+    <mergeCell ref="C89:E89"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="C88:E88"/>
     <mergeCell ref="C64:E64"/>
     <mergeCell ref="C35:E35"/>
     <mergeCell ref="C63:E63"/>
+    <mergeCell ref="C85:E85"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -33185,7 +33566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -34595,6 +34976,41 @@
         </is>
       </c>
       <c r="G48" s="22" t="inlineStr">
+        <is>
+          <t>Roadmap - Open Items &amp; Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="120" customHeight="1">
+      <c r="A49" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="B49" s="39" t="inlineStr">
+        <is>
+          <t>AoE IV-style click-drag wall system (4-session epic)</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>User-requested feature</t>
+        </is>
+      </c>
+      <c r="D49" s="53" t="inlineStr">
+        <is>
+          <t>[~] Partial</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="inlineStr">
+        <is>
+          <t>Session A (free-angle drag-placement of the existing Wall segment) closed 2026-09-16 - see CLAUDE.md's matching status entry. Session B (auto-tiling corner/end-cap pieces, min-3-segment build rule) is blocked on art: corner/end-cap Gemini-&gt;Meshy prompts for all 3 shared pre-Imperial tiers (Ancient/Classical/Durg) plus all 5 civs' Imperial tier are in the 'Art Generation Prompts' sheet (Wall System Session B section, added 2026-09-16). User-supplied corner reference renders confirmed the Classical/Durg style briefs are correct. Open question flagged in that sheet: the corner mesh's own pillar/post region may be extractable and reusable directly as the End-Cap piece (matching AoE's real Pillar+Plank convention) - confirm once the real Meshy geometry is in hand before generating the separate End-Cap images. Session C (gate-interlocking - a Gate placed over a wall line absorbs the overlapping segments and inserts junction pieces) and Session D (a vertex-shader/progress-driven construction-rise visual, replacing ConstructionSite's current scale-squash animation - fully independent of A/B/C, could be done anytime) remain unstarted.</t>
+        </is>
+      </c>
+      <c r="F49" s="22" t="inlineStr">
+        <is>
+          <t>CLAUDE.md / Art Generation Prompts sheet</t>
+        </is>
+      </c>
+      <c r="G49" s="22" t="inlineStr">
         <is>
           <t>Roadmap - Open Items &amp; Priority</t>
         </is>

</xml_diff>

<commit_message>
Wire shared gearless combat body + Classical-tier gear attachment
Corrected the Art Generation Prompts sheet's new-unit sourcing logic:
Skirmisher/Maharaja prompts baked helmet/shield/weapon onto the body,
defeating the per-civ gear-attachment system. Fixed both prompts to
gearless bodies, restructured Maharaja into one shared body + a
per-civ Royal-tier gear row, and set the gear table's Ancient tier to
weapon-only. Saved the underlying AoE modular-construction/rigging
convention to memory.

Built and verified the actual pipeline against user-supplied assets:
decimated a 6,515-tri infantry body to 2,199 tris (bone weights/
bindposes preserved), built a Humanoid Avatar via the existing
HumanoidGltfRigImporter bone map, and wired the 3-piece Classical
gear set via WeaponAttachment.AttachToBone. Live-verified retargeting
and gear placement through the real HumanModelFactory spawn path;
590/590 EditMode tests pass.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KingdomsOfBharat_Master_Reference.xlsx
+++ b/docs/KingdomsOfBharat_Master_Reference.xlsx
@@ -32262,12 +32262,12 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>Simple leather/quilted skull-cap, no metal</t>
+          <t>None - no helmet equipped at this age (bare head)</t>
         </is>
       </c>
       <c r="C18" s="22" t="inlineStr">
         <is>
-          <t>Plain wood-and-hide round shield, unpainted</t>
+          <t>None - no shield equipped at this age (empty off-hand)</t>
         </is>
       </c>
       <c r="D18" s="22" t="inlineStr">
@@ -32277,7 +32277,7 @@
       </c>
       <c r="E18" s="22" t="inlineStr">
         <is>
-          <t>a basic soldier's equipment set for the earliest age, deliberately plain and generic - no civ ornamentation: simple leather/quilted skull-cap, plain wood-and-hide round shield with no markings, unadorned iron short sword or spearhead with plain wood haft, three separate equippable game-asset pieces on a plain background, front and side view each.</t>
+          <t>CORRECTED 2026-09-17 (progressive gear unlock, shared tiers only - Durg/Imperial civ-specific rows below are unaffected): at Ancient age a soldier is equipped with a WEAPON ONLY - bare head, empty off-hand, no helmet or shield exists yet at this tier. Source only one prop: an unadorned iron short sword or spearhead with a plain wood haft, on a plain background, front and side view. Do not generate an Ancient-tier helmet or shield - they are not equipped until Classical (helmet) and remain absent until civ-specific Durg gear introduces a shield (see row below - Classical keeps its own shield as already specified, this rule only removes Ancient's).</t>
         </is>
       </c>
     </row>
@@ -32621,7 +32621,7 @@
       </c>
       <c r="C33" s="22" t="inlineStr">
         <is>
-          <t>a lean, fast South Asian riding horse with simple saddle/bridle/lightweight saddle-cloth, no rider, standing neutral pose, all four legs visible, front view, orthographic. [STATUS: not sourced, reuses shared Cavalry horse]</t>
+          <t>a bare, GEARLESS lean/fast South Asian riding horse - plain coat, no saddle-cloth ornamentation or civ markings baked onto the mesh, bare tack only (a simple neutral bridle/girth strap modeled as part of the horse is fine since it carries no civ identity) - any saddle-cloth, barding, or civ-colored tack accent is a separate attachable prop (reins/chest/head socket points), not part of this body. No rider. Standing neutral pose, all four legs visible, front view, orthographic. [STATUS: not sourced, this is the ONE shared mount reused by Scout, Cavalry, Cavalry Archer, Rajput Royal Guard, and Maratha Mavla Raider - only the rider mesh/gear on top changes per unit]</t>
         </is>
       </c>
     </row>
@@ -32672,7 +32672,7 @@
       </c>
       <c r="C36" s="22" t="inlineStr">
         <is>
-          <t>a swift, lightly-armored South Asian riding horse suited for a mounted archer, no rider, neutral pose, front view, orthographic. [STATUS: not sourced, reuses shared Cavalry horse + Bow prop]</t>
+          <t>reuses the identical shared Cavalry horse mount from row above (Scout) - do not source a second horse model. The mounted-archer look comes entirely from the rider's own gearless body + a bow prop attached to the rider's hand socket, not from a different horse. [STATUS: not sourced as a separate asset - shares the Scout/Cavalry horse mount, differs only by rider + attached Bow prop]</t>
         </is>
       </c>
     </row>
@@ -32689,7 +32689,7 @@
       </c>
       <c r="C37" s="22" t="inlineStr">
         <is>
-          <t>a South Asian riding camel in desert/arid-region tack, simple saddle, no rider, neutral pose, front view, orthographic. [STATUS: not sourced, reuses shared Cavalry+Spearman props]</t>
+          <t>a bare, GEARLESS South Asian riding camel, plain coat and bare tack only (a simple neutral bridle/girth strap modeled as part of the camel is fine since it carries no civ identity) - no saddle-cloth ornamentation, blanket pattern, or civ-colored tack baked onto the mesh; any civ accent belongs on the rider's own per-civ gear, not the mount. No rider. Standing neutral pose, all four legs visible, front view, orthographic. [STATUS: not sourced - a second shared mount, distinct from the Cavalry horse, used only by Camel Rider]</t>
         </is>
       </c>
     </row>
@@ -32815,7 +32815,8 @@
     <row r="45">
       <c r="A45" s="59" t="inlineStr">
         <is>
-          <t>RULE (corrected 2026-09-16): every new-unit HUMAN CHARACTER body (e.g. Skirmisher above, and the Maharaja hero below) must be sourced GEARLESS - no helmet, shield, or weapon baked onto the mesh. Helmet/shield/weapon are always separate equippable props attached at runtime via bone sockets (WeaponAttachment.AttachToBone), per the 'Per-civ unit gear' table above. Mount-only/machine-only/hull-only assets (Scout horse, Battering Ram, Scorpion, Fire Ship, etc.) are unaffected - they carry no character gear at all.</t>
+          <t>RULE (corrected 2026-09-16): every new-unit HUMAN CHARACTER body (e.g. Skirmisher above, and the Maharaja hero below) must be sourced GEARLESS - no helmet, shield, or weapon baked onto the mesh. Helmet/shield/weapon are always separate equippable props attached at runtime via bone sockets (WeaponAttachment.AttachToBone), per the 'Per-civ unit gear' table above. Mount-only/machine-only/hull-only assets (Scout horse, Battering Ram, Scorpion, Fire Ship, etc.) are unaffected - they carry no character gear at all.
+The same rule extends to MOUNTS: no saddle-cloth/barding/civ ornamentation baked onto a horse or camel body - any civ-colored tack or barding is a separate attachable prop, exactly like rider gear. AUDIT FLAG (not yet verified either way): the existing Maurya/Vijayanagara War Elephant models predate this rule and were never checked for whether their howdah/mahout platform is a separate mesh from the elephant body - re-verify before assuming they already comply, and re-source with a bare-elephant-body prompt (elephant only, no howdah/armor baked on, mahout rider reusing the shared humanoid body, howdah as its own separate attachable structure) if they don't.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Relics + Monastery collection (Wave 6 item 35)
Economic-only, no new victory condition, per the 2026-09-15 design
decision. New Relic (neutral world prop) and RelicCarrier (walk/pick-up/
auto-deliver to the nearest owned Monastery, mirroring Trader's own
state-machine shape) - added to every land unit factory that already
carries GarrisonSeeker. Monastery gains a relic count and a passive Gold
trickle. Relics spawn on the map via ResourceNodeSpawner. Live-verified
end to end via UnityMCP: pickup, auto-walk, deposit, gold trickle, and
death-drop all confirmed through the real production path.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KingdomsOfBharat_Master_Reference.xlsx
+++ b/docs/KingdomsOfBharat_Master_Reference.xlsx
@@ -30296,6 +30296,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -30306,7 +30307,7 @@
     <row r="5" ht="74" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Waves 0 through 5 of docs/IMPLEMENTATION_ROADMAP.md are ALL CLOSED (2026-09-04 to 2026-09-14). Wave 6 - the parallel-safe economy/meta backlog - is the only open wave; 5 of its 9 items (Town Bell, idle-worker indicator, cheat codes, Score system, tutorial content) are done - every decision-free item is now closed. The AoE-parity plan's Phases 1-4 are resolved and Phase 5 (multiplayer) is complete except for testing that needs a second physical machine. Remaining Wave 6 items (Relics, Wonder/KotH victory conditions, game modes) all need a design decision first; otherwise development is a long tail of UI/art polish and asset sourcing.</t>
+          <t>Waves 0 through 5 of docs/IMPLEMENTATION_ROADMAP.md are ALL CLOSED (2026-09-04 to 2026-09-14). Wave 6 - the parallel-safe economy/meta backlog - is the only open wave; 6 of its 9 items (Town Bell, idle-worker indicator, cheat codes, Score system, tutorial content, Relics + Monastery collection) are done. The AoE-parity plan's Phases 1-4 are resolved and Phase 5 (multiplayer) is complete except for testing that needs a second physical machine. Remaining Wave 6 items (Relics, Wonder/KotH victory conditions, game modes) all need a design decision first; otherwise development is a long tail of UI/art polish and asset sourcing.</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -30315,6 +30316,7 @@
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="6" t="n"/>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
@@ -30534,10 +30536,11 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>OPEN. Items 33 (Town Bell) and 34 (idle-worker indicator) closed 2026-09-14. Remaining: Relics + relic storage (35), Score system (36), Wonder/Relic victory conditions (37), game modes (38), cheat codes (39), tutorial content (40), soundtrack.</t>
-        </is>
-      </c>
-    </row>
+          <t>OPEN. Items 33, 34, 36, 39, 40 and 35 (Relics + Monastery collection, closed 2026-09-17) are done. Remaining: Wonder/Relic victory conditions (37, King of the Hill half still open), game modes (38, Deathmatch + King of the Hill), soundtrack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
@@ -30677,6 +30680,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
@@ -30808,6 +30812,7 @@
         <v/>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
@@ -30871,6 +30876,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
@@ -30895,6 +30901,7 @@
     <row r="48" ht="44" customHeight="1">
       <c r="A48" s="22" t="n"/>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
@@ -31106,6 +31113,7 @@
         </is>
       </c>
     </row>
+    <row r="63"/>
     <row r="64" ht="32" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
@@ -31137,6 +31145,7 @@
     <row r="68">
       <c r="A68" s="22" t="n"/>
     </row>
+    <row r="69"/>
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
@@ -31147,7 +31156,7 @@
     <row r="71">
       <c r="A71" s="22" t="inlineStr">
         <is>
-          <t>The project's own session protocol is one roadmap item per session, user's call on which. As of 2026-09-15, every decision-free Wave 6 item is closed (Town Bell, idle-worker indicator, cheat codes, Score system, Tutorial content), AND the Relics/Wonder/game-modes design decision is now resolved (Relics+Monastery economic-only, Deathmatch, King of the Hill; Wonder declined). Age-tiered building mesh decimation (the last flagged follow-up from the 2026-09-15 regression fix) closed 2026-09-16. What's left: (1) implement Relics + Monastery collection (35); (2) implement Deathmatch mode (38); (3) implement King of the Hill zone-control victory (37/38); (4) unit-side team colour once Blender masks are sourced; (5) UI/art polish or further balance passes, user's call.</t>
+          <t>The project's own session protocol is one roadmap item per session, user's call on which. Relics + Monastery collection (35) closed 2026-09-17. What's left: (1) implement Deathmatch mode (38); (2) implement King of the Hill zone-control victory (37/38); (3) unit-side team colour once Blender masks are sourced; (4) UI/art polish or further balance passes, user's call.</t>
         </is>
       </c>
     </row>
@@ -37063,12 +37072,12 @@
       </c>
       <c r="F39" s="56" t="inlineStr">
         <is>
-          <t>[ ] Not Started</t>
+          <t>[OK] Implemented</t>
         </is>
       </c>
       <c r="G39" s="22" t="inlineStr">
         <is>
-          <t>DESIGN DECISION RESOLVED 2026-09-15 via AskUserQuestion: build it, economic only. Relics spawn on the map (or drop from destroyed scripted targets), carried by any land unit to a Monastery for a passive Gold trickle (AoE II precedent: 0.5-1x gold/sec per relic garrisoned). Explicitly NO new victory condition tied to relic count/ownership - stays purely economic, keeping scope smaller (user chose "Economic only" over "also add a Relic-count victory option" via AskUserQuestion). Monastery (Wave 4 item 27) is the existing carrier building - no new building needed. Not yet implemented - this was a design-decision-only session, not implementation.</t>
+          <t>Closed 2026-09-17. Implemented per the 2026-09-15 design decision: economic only, no new victory condition. New Resources/Relic.cs (neutral world prop, held/unheld flag) and Resources/RelicCarrier.cs (added to every land unit factory that already carries GarrisonSeeker - 20 factories - mirroring that item's own broad-add convention): right-click an unclaimed Relic picks it up (reparented onto the carrying unit, no dedicated carried-Relic art exists yet - flagged per the flag-asset-needs convention), auto-routes to the nearest owned Monastery (FindNearestOwnedMonastery, same shape as Trader.FindNearestOwnedMarket), and deposits automatically on arrival - a one-shot pickup-then-deliver, not an endless shuttle like Trader. A carrier that dies mid-carry drops the Relic at its death position (RelicCarrier.OnDestroy unparents it, live-verified). Monastery.cs gained RelicCount/AddRelic()/a passive Gold trickle (0.5 Gold/sec/Relic while complete, first-pass rate, not independently balanced, same disclosed convention as Trader's own ComputeTradeGold) via a new internal Tick(deltaTime) (Farm.Tick's own testability convention) and a pure RelicGoldPerTick formula. Relics spawn on the map via ResourceNodeSpawner.SpawnRelic (reuses its existing RNG/ring-placement convention; new MapDefinitionData.RelicCount=5 on every map, deliberately NOT scaled with map area like resource counts - Relics stay scarce regardless of map size). SelectionManager gained a hitRelic branch (neutral, no friendly-gate - any faction's unit can grab it first, matching AoE's own rule) plus CancelCarry() wired into every other order branch's cancel chain. 10 new EditMode tests (RelicTests.cs: held-state flag, FindNearestOwnedMonastery routing, RelicGoldPerTick formula, Monastery.Tick gold-trickle behavior - 601/601 total, up from 591, all pass). Live-verified via UnityMCP through the real production path: a real match (5 real Relics spawned on RiverValley, matching RelicCount), a real Monastery placed and completed, a real Player Worker's RelicCarrier.PickUp() reparented the Relic onto it (IsHeld=true, parent=Worker); left to run through its own real Update()/NavMeshAgent loop with no further intervention, the worker auto-walked ~38 units to the Monastery and deposited on its own (Monastery.RelicCount 0-&gt;1, Relic GameObject destroyed, 4 Relics remained in the scene); the real Player Gold stockpile was independently confirmed climbing on its own between two unrelated tool calls (17.6 -&gt; 21.0 -&gt; 24.2 over consecutive real wall-clock gaps, consistent with 0.5 Gold/sec for 1 held Relic and no other active Gold source in that match) - the live gold-trickle Update() loop, not just the isolated unit test. Separately live-verified the death-drop case: picked up a second Relic, destroyed the carrying Worker mid-route, and confirmed the Relic correctly reappeared unparented and IsHeld=false at the Worker's exact death position. Full EditMode suite re-confirmed 601/601 after exiting Play mode. No AI-side use of Relics (no AI pickup/delivery hook) - new capability, not existing behavior moved, matching every other Wave 4/6 item's own precedent for skipping the AI hook without calling it a regression.</t>
         </is>
       </c>
       <c r="H39" s="22" t="inlineStr">

</xml_diff>